<commit_message>
feat: Generate NBA predictions, implement cache statistics tracking, and remove unused CSS.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-14.xlsx
+++ b/results/nba_predictions_2025-12-14.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>46.15</v>
+        <v>58.84</v>
       </c>
       <c r="E2" t="n">
-        <v>53.85</v>
+        <v>41.16</v>
       </c>
       <c r="F2" t="n">
-        <v>59.57</v>
+        <v>59.62</v>
       </c>
       <c r="G2" t="n">
-        <v>40.43</v>
+        <v>40.38</v>
       </c>
       <c r="H2" t="n">
         <v>-0.33</v>
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -608,13 +608,13 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>46.2</v>
+        <v>58.8</v>
       </c>
       <c r="S2" t="n">
-        <v>53.8</v>
+        <v>41.2</v>
       </c>
       <c r="T2" t="n">
-        <v>235.7</v>
+        <v>230.2</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>-2.3</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="3">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>39</v>
+        <v>57.81</v>
       </c>
       <c r="E3" t="n">
-        <v>61</v>
+        <v>42.19</v>
       </c>
       <c r="F3" t="n">
-        <v>59.16</v>
+        <v>59.2</v>
       </c>
       <c r="G3" t="n">
-        <v>40.84</v>
+        <v>40.8</v>
       </c>
       <c r="H3" t="n">
         <v>0.09</v>
@@ -693,13 +693,13 @@
         <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>39</v>
+        <v>57.8</v>
       </c>
       <c r="S3" t="n">
-        <v>61</v>
+        <v>42.2</v>
       </c>
       <c r="T3" t="n">
-        <v>229.3</v>
+        <v>211.6</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -708,7 +708,7 @@
       </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="n">
-        <v>-6.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="4">
@@ -728,16 +728,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>39</v>
+        <v>57.81</v>
       </c>
       <c r="E4" t="n">
-        <v>61</v>
+        <v>42.19</v>
       </c>
       <c r="F4" t="n">
-        <v>57.01</v>
+        <v>56.9</v>
       </c>
       <c r="G4" t="n">
-        <v>42.99</v>
+        <v>43.1</v>
       </c>
       <c r="H4" t="n">
         <v>-0.19</v>
@@ -774,13 +774,13 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>39</v>
+        <v>57.8</v>
       </c>
       <c r="S4" t="n">
-        <v>61</v>
+        <v>42.2</v>
       </c>
       <c r="T4" t="n">
-        <v>230.2</v>
+        <v>223.8</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>-6.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="5">
@@ -809,16 +809,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>54.35</v>
+        <v>54.4</v>
       </c>
       <c r="G5" t="n">
-        <v>45.65</v>
+        <v>45.6</v>
       </c>
       <c r="H5" t="n">
         <v>-0.84</v>
@@ -840,7 +840,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -855,13 +855,13 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="S5" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="T5" t="n">
-        <v>225.6</v>
+        <v>223.9</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>-6.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -894,16 +894,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>57.81</v>
       </c>
       <c r="E6" t="n">
-        <v>61</v>
+        <v>42.19</v>
       </c>
       <c r="F6" t="n">
-        <v>58.67</v>
+        <v>58.65</v>
       </c>
       <c r="G6" t="n">
-        <v>41.33</v>
+        <v>41.35</v>
       </c>
       <c r="H6" t="n">
         <v>-0.04</v>
@@ -940,13 +940,13 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>39</v>
+        <v>57.8</v>
       </c>
       <c r="S6" t="n">
-        <v>61</v>
+        <v>42.2</v>
       </c>
       <c r="T6" t="n">
-        <v>226.2</v>
+        <v>202.6</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="W6" t="n">
-        <v>-6.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="7">
@@ -979,16 +979,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>60.71</v>
+        <v>70.59</v>
       </c>
       <c r="E7" t="n">
-        <v>39.29</v>
+        <v>29.41</v>
       </c>
       <c r="F7" t="n">
-        <v>57.36</v>
+        <v>57.33</v>
       </c>
       <c r="G7" t="n">
-        <v>42.64</v>
+        <v>42.67</v>
       </c>
       <c r="H7" t="n">
         <v>-0.43</v>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1025,13 +1025,13 @@
         <v>-0</v>
       </c>
       <c r="R7" t="n">
-        <v>60.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="S7" t="n">
-        <v>39.3</v>
+        <v>29.4</v>
       </c>
       <c r="T7" t="n">
-        <v>238.2</v>
+        <v>236</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="W7" t="n">
-        <v>6.4</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="8">
@@ -1064,16 +1064,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>39</v>
+        <v>57.81</v>
       </c>
       <c r="E8" t="n">
-        <v>61</v>
+        <v>42.19</v>
       </c>
       <c r="F8" t="n">
-        <v>56.66</v>
+        <v>56.65</v>
       </c>
       <c r="G8" t="n">
-        <v>43.34</v>
+        <v>43.35</v>
       </c>
       <c r="H8" t="n">
         <v>-0.35</v>
@@ -1110,17 +1110,17 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>39</v>
+        <v>57.8</v>
       </c>
       <c r="S8" t="n">
-        <v>61</v>
+        <v>42.2</v>
       </c>
       <c r="T8" t="n">
-        <v>227.2</v>
+        <v>219.7</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Devin Booker (QUESTIONABLE)</t>
+          <t>Devin Booker (AVAILABLE)</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="W8" t="n">
-        <v>-6.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="9">
@@ -1149,16 +1149,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E9" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>56.26</v>
+        <v>56.33</v>
       </c>
       <c r="G9" t="n">
-        <v>43.74</v>
+        <v>43.67</v>
       </c>
       <c r="H9" t="n">
         <v>-0.28</v>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1195,17 +1195,17 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="S9" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="T9" t="n">
-        <v>228.1</v>
+        <v>217.1</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Donovan Clingan (QUESTIONABLE)</t>
+          <t>Donovan Clingan (AVAILABLE)</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="W9" t="n">
-        <v>-6.6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add advanced ML features, database maintenance scripts, process management, and update Docker environment with new caching.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-14.xlsx
+++ b/results/nba_predictions_2025-12-14.xlsx
@@ -568,10 +568,10 @@
         <v>41.16</v>
       </c>
       <c r="F2" t="n">
-        <v>59.62</v>
+        <v>59.57</v>
       </c>
       <c r="G2" t="n">
-        <v>40.38</v>
+        <v>40.43</v>
       </c>
       <c r="H2" t="n">
         <v>-0.33</v>
@@ -653,10 +653,10 @@
         <v>42.19</v>
       </c>
       <c r="F3" t="n">
-        <v>59.2</v>
+        <v>59.24</v>
       </c>
       <c r="G3" t="n">
-        <v>40.8</v>
+        <v>40.76</v>
       </c>
       <c r="H3" t="n">
         <v>0.09</v>
@@ -815,10 +815,10 @@
         <v>50</v>
       </c>
       <c r="F5" t="n">
-        <v>54.4</v>
+        <v>54.42</v>
       </c>
       <c r="G5" t="n">
-        <v>45.6</v>
+        <v>45.58</v>
       </c>
       <c r="H5" t="n">
         <v>-0.84</v>
@@ -900,10 +900,10 @@
         <v>42.19</v>
       </c>
       <c r="F6" t="n">
-        <v>58.65</v>
+        <v>58.68</v>
       </c>
       <c r="G6" t="n">
-        <v>41.35</v>
+        <v>41.32</v>
       </c>
       <c r="H6" t="n">
         <v>-0.04</v>
@@ -985,10 +985,10 @@
         <v>29.41</v>
       </c>
       <c r="F7" t="n">
-        <v>57.33</v>
+        <v>57.39</v>
       </c>
       <c r="G7" t="n">
-        <v>42.67</v>
+        <v>42.61</v>
       </c>
       <c r="H7" t="n">
         <v>-0.43</v>
@@ -1070,10 +1070,10 @@
         <v>42.19</v>
       </c>
       <c r="F8" t="n">
-        <v>56.65</v>
+        <v>56.71</v>
       </c>
       <c r="G8" t="n">
-        <v>43.35</v>
+        <v>43.29</v>
       </c>
       <c r="H8" t="n">
         <v>-0.35</v>
@@ -1155,10 +1155,10 @@
         <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>56.33</v>
+        <v>56.28</v>
       </c>
       <c r="G9" t="n">
-        <v>43.67</v>
+        <v>43.72</v>
       </c>
       <c r="H9" t="n">
         <v>-0.28</v>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Seth Curry (QUESTIONABLE)</t>
+          <t>Seth Curry (AVAILABLE)</t>
         </is>
       </c>
       <c r="W9" t="n">

</xml_diff>